<commit_message>
live google excel leads
</commit_message>
<xml_diff>
--- a/sample lead data.xlsx
+++ b/sample lead data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MOTHAN\crm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\crm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AD82EAB-16D6-4ABB-99E9-4C2A4577F75A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{37184E61-8101-4040-B05E-75A9DA179214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{FEE06FA0-051F-4B10-AB00-81C3D305DED1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FEE06FA0-051F-4B10-AB00-81C3D305DED1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="71">
   <si>
     <t xml:space="preserve"> Enq no</t>
   </si>
@@ -214,6 +214,39 @@
   </si>
   <si>
     <t>Parking</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>vijay@gmail.com</t>
+  </si>
+  <si>
+    <t>Anub Kumar Gain@gmail.com</t>
+  </si>
+  <si>
+    <t>Hameed@gmail.com</t>
+  </si>
+  <si>
+    <t>Manikandan@gmail.com</t>
+  </si>
+  <si>
+    <t>Bhuvanesh@gmail.com</t>
+  </si>
+  <si>
+    <t>Mohith Manjunath@gmail.com</t>
+  </si>
+  <si>
+    <t>JayanthiVinoth@gmail.com</t>
+  </si>
+  <si>
+    <t>ShakeelMohammed@gmail.com</t>
+  </si>
+  <si>
+    <t>NagendranRajaPradeep@gmail.com</t>
+  </si>
+  <si>
+    <t>kumarappan@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -223,7 +256,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -252,6 +285,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -301,10 +342,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -336,8 +378,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -684,7 +730,9 @@
       <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2"/>
+      <c r="J1" s="8" t="s">
+        <v>60</v>
+      </c>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
@@ -734,6 +782,9 @@
       <c r="I2" s="10" t="s">
         <v>13</v>
       </c>
+      <c r="J2" s="11" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="3" spans="1:31" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="9">
@@ -763,6 +814,9 @@
       <c r="I3" s="10" t="s">
         <v>19</v>
       </c>
+      <c r="J3" s="11" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="4" spans="1:31" s="9" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
@@ -792,6 +846,9 @@
       <c r="I4" s="10" t="s">
         <v>22</v>
       </c>
+      <c r="J4" s="11" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="5" spans="1:31" s="10" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="10">
@@ -821,6 +878,9 @@
       <c r="I5" s="10" t="s">
         <v>29</v>
       </c>
+      <c r="J5" s="11" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="6" spans="1:31" s="10" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="10">
@@ -850,6 +910,9 @@
       <c r="I6" s="10" t="s">
         <v>32</v>
       </c>
+      <c r="J6" s="11" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="7" spans="1:31" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
@@ -879,6 +942,9 @@
       <c r="I7" s="10" t="s">
         <v>39</v>
       </c>
+      <c r="J7" s="11" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="8" spans="1:31" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
@@ -908,6 +974,9 @@
       <c r="I8" s="10" t="s">
         <v>39</v>
       </c>
+      <c r="J8" s="11" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="9" spans="1:31" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
@@ -937,6 +1006,9 @@
       <c r="I9" s="10" t="s">
         <v>51</v>
       </c>
+      <c r="J9" s="11" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="10" spans="1:31" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
@@ -966,6 +1038,9 @@
       <c r="I10" s="10" t="s">
         <v>55</v>
       </c>
+      <c r="J10" s="11" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="11" spans="1:31" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="9">
@@ -995,9 +1070,22 @@
       <c r="I11" s="10" t="s">
         <v>59</v>
       </c>
+      <c r="J11" s="11" t="s">
+        <v>66</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="J2" r:id="rId1" xr:uid="{D0945B20-2D52-454C-8EF8-DE3E6FDF2EEB}"/>
+    <hyperlink ref="J4" r:id="rId2" xr:uid="{8CDC1C61-431F-49A2-B248-D0295224F0FE}"/>
+    <hyperlink ref="J7" r:id="rId3" xr:uid="{5CED1F62-4E50-4061-95C8-BA71F412F571}"/>
+    <hyperlink ref="J8" r:id="rId4" xr:uid="{C3758DC6-E3F6-481D-9CD7-BA332BBF1B05}"/>
+    <hyperlink ref="J9" r:id="rId5" xr:uid="{C3B8D31E-1848-49CF-8995-A8E5573E37C0}"/>
+    <hyperlink ref="J10" r:id="rId6" xr:uid="{F2BB6A25-C152-49CC-9441-95D8E91E340D}"/>
+    <hyperlink ref="J6" r:id="rId7" xr:uid="{91569912-BEA2-43B5-9592-4C9009346DBC}"/>
+    <hyperlink ref="J5" r:id="rId8" xr:uid="{373F89A4-A47B-4077-9AD1-3782B8DD842F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>